<commit_message>
Agregado indice asociado a las estaciones de carga
</commit_message>
<xml_diff>
--- a/data/data_electrico_var_3turnos_chuqui_seasons/elmo_data.xlsx
+++ b/data/data_electrico_var_3turnos_chuqui_seasons/elmo_data.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\ELMO\Modelos\Old_models\ELMO-UG-Paper_noswap\data\data_electrico_var_3turnos_chuqui_seasons\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\ELMO-UG-Paper\data\data_electrico_var_3turnos_chuqui_seasons\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66465CBB-382F-4501-976D-2804D1046404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE38937-AC59-4ED2-9F1C-0C3ADA4776F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="3300" windowWidth="16800" windowHeight="9750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
     <sheet name="LHD" sheetId="2" r:id="rId2"/>
-    <sheet name="extraction_nodes" sheetId="3" r:id="rId3"/>
-    <sheet name="discharge_nodes" sheetId="4" r:id="rId4"/>
+    <sheet name="stations" sheetId="5" r:id="rId3"/>
+    <sheet name="extraction_nodes" sheetId="3" r:id="rId4"/>
+    <sheet name="discharge_nodes" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="125">
   <si>
     <t>id</t>
   </si>
@@ -381,6 +382,36 @@
   </si>
   <si>
     <t>Profile_Chuquicamata</t>
+  </si>
+  <si>
+    <t>station_name</t>
+  </si>
+  <si>
+    <t>station_cost</t>
+  </si>
+  <si>
+    <t>distance_to_dn</t>
+  </si>
+  <si>
+    <t>max_chargers</t>
+  </si>
+  <si>
+    <t>man_time</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>station_1</t>
+  </si>
+  <si>
+    <t>station_2</t>
+  </si>
+  <si>
+    <t>station_3</t>
   </si>
 </sst>
 </file>
@@ -1235,24 +1266,24 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AC34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.7265625" style="32" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" style="17" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.54296875" style="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.1796875" style="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="33" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" style="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.77734375" style="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" style="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" style="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.21875" style="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" style="17" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="17" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.453125" style="33" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="33" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.44140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -1303,7 +1334,7 @@
       <c r="AB1" s="36"/>
       <c r="AC1" s="36"/>
     </row>
-    <row r="2" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="40" t="s">
         <v>3</v>
       </c>
@@ -1354,7 +1385,7 @@
       <c r="AB2" s="36"/>
       <c r="AC2" s="36"/>
     </row>
-    <row r="3" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41">
         <v>1</v>
       </c>
@@ -1405,7 +1436,7 @@
       <c r="AB3" s="46"/>
       <c r="AC3" s="46"/>
     </row>
-    <row r="4" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="41">
         <v>2</v>
       </c>
@@ -1456,7 +1487,7 @@
       <c r="AB4" s="46"/>
       <c r="AC4" s="46"/>
     </row>
-    <row r="5" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="41">
         <v>3</v>
       </c>
@@ -1507,7 +1538,7 @@
       <c r="AB5" s="46"/>
       <c r="AC5" s="46"/>
     </row>
-    <row r="6" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="41">
         <v>4</v>
       </c>
@@ -1558,7 +1589,7 @@
       <c r="AB6" s="46"/>
       <c r="AC6" s="46"/>
     </row>
-    <row r="7" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="41"/>
       <c r="B7" s="43"/>
       <c r="C7" s="45"/>
@@ -1573,7 +1604,7 @@
       <c r="L7" s="52"/>
       <c r="M7" s="52"/>
     </row>
-    <row r="8" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="41"/>
       <c r="B8" s="43"/>
       <c r="C8" s="45"/>
@@ -1588,7 +1619,7 @@
       <c r="L8" s="52"/>
       <c r="M8" s="52"/>
     </row>
-    <row r="9" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="41"/>
       <c r="B9" s="43"/>
       <c r="C9" s="45"/>
@@ -1603,7 +1634,7 @@
       <c r="L9" s="52"/>
       <c r="M9" s="52"/>
     </row>
-    <row r="10" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="41"/>
       <c r="B10" s="43"/>
       <c r="C10" s="45"/>
@@ -1618,7 +1649,7 @@
       <c r="L10" s="52"/>
       <c r="M10" s="52"/>
     </row>
-    <row r="11" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="41"/>
       <c r="B11" s="43"/>
       <c r="C11" s="45"/>
@@ -1633,7 +1664,7 @@
       <c r="L11" s="52"/>
       <c r="M11" s="52"/>
     </row>
-    <row r="12" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="41"/>
       <c r="B12" s="43"/>
       <c r="C12" s="45"/>
@@ -1648,7 +1679,7 @@
       <c r="L12" s="52"/>
       <c r="M12" s="52"/>
     </row>
-    <row r="13" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="41"/>
       <c r="B13" s="43"/>
       <c r="C13" s="45"/>
@@ -1663,7 +1694,7 @@
       <c r="L13" s="52"/>
       <c r="M13" s="52"/>
     </row>
-    <row r="14" spans="1:29" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:29" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="41"/>
       <c r="B14" s="43"/>
       <c r="C14" s="45"/>
@@ -1678,7 +1709,7 @@
       <c r="L14" s="52"/>
       <c r="M14" s="52"/>
     </row>
-    <row r="15" spans="1:29" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:29" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="41"/>
       <c r="B15" s="43"/>
       <c r="C15" s="45"/>
@@ -1693,7 +1724,7 @@
       <c r="L15" s="52"/>
       <c r="M15" s="52"/>
     </row>
-    <row r="16" spans="1:29" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:29" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="41"/>
       <c r="B16" s="43"/>
       <c r="C16" s="45"/>
@@ -1708,7 +1739,7 @@
       <c r="L16" s="52"/>
       <c r="M16" s="52"/>
     </row>
-    <row r="17" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="41"/>
       <c r="B17" s="43"/>
       <c r="C17" s="45"/>
@@ -1723,7 +1754,7 @@
       <c r="L17" s="52"/>
       <c r="M17" s="52"/>
     </row>
-    <row r="18" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="41"/>
       <c r="B18" s="43"/>
       <c r="C18" s="45"/>
@@ -1738,7 +1769,7 @@
       <c r="L18" s="52"/>
       <c r="M18" s="52"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="41"/>
       <c r="B19" s="43"/>
       <c r="C19" s="45"/>
@@ -1753,7 +1784,7 @@
       <c r="L19" s="52"/>
       <c r="M19" s="52"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="41"/>
       <c r="B20" s="43"/>
       <c r="C20" s="45"/>
@@ -1768,7 +1799,7 @@
       <c r="L20" s="52"/>
       <c r="M20" s="52"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="41"/>
       <c r="B21" s="43"/>
       <c r="C21" s="45"/>
@@ -1783,7 +1814,7 @@
       <c r="L21" s="52"/>
       <c r="M21" s="52"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="41"/>
       <c r="B22" s="43"/>
       <c r="C22" s="45"/>
@@ -1798,7 +1829,7 @@
       <c r="L22" s="52"/>
       <c r="M22" s="52"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="41"/>
       <c r="B23" s="43"/>
       <c r="C23" s="45"/>
@@ -1813,7 +1844,7 @@
       <c r="L23" s="52"/>
       <c r="M23" s="52"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="41"/>
       <c r="B24" s="43"/>
       <c r="C24" s="45"/>
@@ -1828,7 +1859,7 @@
       <c r="L24" s="52"/>
       <c r="M24" s="52"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="41"/>
       <c r="B25" s="43"/>
       <c r="C25" s="45"/>
@@ -1843,7 +1874,7 @@
       <c r="L25" s="52"/>
       <c r="M25" s="52"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="41"/>
       <c r="B26" s="43"/>
       <c r="C26" s="45"/>
@@ -1858,7 +1889,7 @@
       <c r="L26" s="52"/>
       <c r="M26" s="52"/>
     </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" s="33"/>
     </row>
   </sheetData>
@@ -1873,36 +1904,35 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AD17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.453125" style="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1796875" style="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.26953125" style="30" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.54296875" style="30" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.453125" style="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" style="30" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" style="30" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" style="30" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.54296875" style="30" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7265625" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.1796875" style="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="30" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.77734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.21875" style="30" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="30" customWidth="1"/>
-    <col min="16" max="16" width="17.1796875" style="30" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5546875" style="31" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="31" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.81640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.81640625" style="31" customWidth="1"/>
-    <col min="24" max="24" width="18.453125" style="31" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.54296875" style="31" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.26953125" style="31" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.77734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.77734375" style="31" customWidth="1"/>
+    <col min="24" max="24" width="18.44140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -1994,7 +2024,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="40" t="s">
         <v>3</v>
       </c>
@@ -2086,7 +2116,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41">
         <v>1</v>
       </c>
@@ -2178,7 +2208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="41">
         <v>2</v>
       </c>
@@ -2270,7 +2300,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="41">
         <v>3</v>
       </c>
@@ -2362,7 +2392,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="41">
         <v>4</v>
       </c>
@@ -2454,7 +2484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="41"/>
       <c r="B7" s="70"/>
       <c r="C7" s="71"/>
@@ -2479,7 +2509,7 @@
       <c r="V7" s="46"/>
       <c r="W7" s="46"/>
     </row>
-    <row r="8" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="41"/>
       <c r="B8" s="43"/>
       <c r="C8" s="45"/>
@@ -2504,7 +2534,7 @@
       <c r="V8" s="46"/>
       <c r="W8" s="46"/>
     </row>
-    <row r="9" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="41"/>
       <c r="B9" s="43"/>
       <c r="C9" s="45"/>
@@ -2529,7 +2559,7 @@
       <c r="V9" s="46"/>
       <c r="W9" s="46"/>
     </row>
-    <row r="10" spans="1:30" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="58"/>
       <c r="B10" s="59"/>
       <c r="C10" s="60"/>
@@ -2554,7 +2584,7 @@
       <c r="V10" s="68"/>
       <c r="W10" s="68"/>
     </row>
-    <row r="11" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="41"/>
       <c r="B11" s="43"/>
       <c r="C11" s="45"/>
@@ -2581,7 +2611,7 @@
       <c r="Z11" s="69"/>
       <c r="AA11" s="69"/>
     </row>
-    <row r="12" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="41"/>
       <c r="B12" s="43"/>
       <c r="C12" s="45"/>
@@ -2608,7 +2638,7 @@
       <c r="Z12" s="69"/>
       <c r="AA12" s="69"/>
     </row>
-    <row r="13" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="41"/>
       <c r="B13" s="43"/>
       <c r="C13" s="45"/>
@@ -2635,7 +2665,7 @@
       <c r="Z13" s="69"/>
       <c r="AA13" s="69"/>
     </row>
-    <row r="14" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:30" s="46" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="41"/>
       <c r="B14" s="43"/>
       <c r="C14" s="45"/>
@@ -2662,9 +2692,9 @@
       <c r="Z14" s="69"/>
       <c r="AA14" s="69"/>
     </row>
-    <row r="15" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="16" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2672,21 +2702,131 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D86F6B0-26ED-4B02-B890-EDAFE42B3137}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3">
+        <v>70000</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4">
+        <v>214000</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5">
+        <v>150000</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H346"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" style="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="13.54296875" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.1796875" style="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.54296875" style="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.5546875" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.21875" style="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2712,7 +2852,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
@@ -2738,7 +2878,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>0</v>
       </c>
@@ -2764,7 +2904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16">
         <v>1</v>
       </c>
@@ -2790,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="16">
         <v>2</v>
       </c>
@@ -2816,7 +2956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
         <v>3</v>
       </c>
@@ -2842,7 +2982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16">
         <v>4</v>
       </c>
@@ -2868,7 +3008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16">
         <v>5</v>
       </c>
@@ -2894,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16">
         <v>6</v>
       </c>
@@ -2920,7 +3060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="16">
         <v>7</v>
       </c>
@@ -2946,7 +3086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16">
         <v>8</v>
       </c>
@@ -2972,7 +3112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16">
         <v>9</v>
       </c>
@@ -2998,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16">
         <v>10</v>
       </c>
@@ -3024,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="16">
         <v>11</v>
       </c>
@@ -3050,7 +3190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16">
         <v>12</v>
       </c>
@@ -3076,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="16">
         <v>13</v>
       </c>
@@ -3102,7 +3242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="16">
         <v>14</v>
       </c>
@@ -3128,7 +3268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="16">
         <v>15</v>
       </c>
@@ -3154,7 +3294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16">
         <v>16</v>
       </c>
@@ -3180,7 +3320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="16">
         <v>17</v>
       </c>
@@ -3206,7 +3346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16">
         <v>18</v>
       </c>
@@ -3232,7 +3372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16">
         <v>19</v>
       </c>
@@ -3258,7 +3398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16">
         <v>20</v>
       </c>
@@ -3284,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="16">
         <v>21</v>
       </c>
@@ -3310,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="16">
         <v>22</v>
       </c>
@@ -3336,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="16">
         <v>23</v>
       </c>
@@ -3362,7 +3502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="16">
         <v>24</v>
       </c>
@@ -3388,7 +3528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="16">
         <v>25</v>
       </c>
@@ -3414,7 +3554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="16">
         <v>26</v>
       </c>
@@ -3440,7 +3580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="16">
         <v>27</v>
       </c>
@@ -3466,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="16">
         <v>28</v>
       </c>
@@ -3492,7 +3632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="16">
         <v>29</v>
       </c>
@@ -3518,7 +3658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16">
         <v>30</v>
       </c>
@@ -3544,7 +3684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="16">
         <v>31</v>
       </c>
@@ -3570,7 +3710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="16">
         <v>32</v>
       </c>
@@ -3596,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="16">
         <v>33</v>
       </c>
@@ -3622,7 +3762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="16">
         <v>34</v>
       </c>
@@ -3648,7 +3788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="16">
         <v>35</v>
       </c>
@@ -3674,7 +3814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="16">
         <v>36</v>
       </c>
@@ -3700,7 +3840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="16">
         <v>37</v>
       </c>
@@ -3726,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="16">
         <v>38</v>
       </c>
@@ -3752,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="16">
         <v>39</v>
       </c>
@@ -3778,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="16"/>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
@@ -3788,7 +3928,7 @@
       <c r="G43" s="16"/>
       <c r="H43" s="14"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="16"/>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
@@ -3798,7 +3938,7 @@
       <c r="G44" s="16"/>
       <c r="H44" s="14"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="16"/>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -3808,7 +3948,7 @@
       <c r="G45" s="16"/>
       <c r="H45" s="14"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="16"/>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
@@ -3818,7 +3958,7 @@
       <c r="G46" s="16"/>
       <c r="H46" s="14"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="16"/>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
@@ -3828,7 +3968,7 @@
       <c r="G47" s="16"/>
       <c r="H47" s="14"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="16"/>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
@@ -3838,7 +3978,7 @@
       <c r="G48" s="16"/>
       <c r="H48" s="14"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="16"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
@@ -3848,7 +3988,7 @@
       <c r="G49" s="16"/>
       <c r="H49" s="14"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="16"/>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -3858,7 +3998,7 @@
       <c r="G50" s="16"/>
       <c r="H50" s="14"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="16"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
@@ -3868,7 +4008,7 @@
       <c r="G51" s="16"/>
       <c r="H51" s="14"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="16"/>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
@@ -3878,7 +4018,7 @@
       <c r="G52" s="16"/>
       <c r="H52" s="14"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="16"/>
       <c r="B53" s="15"/>
       <c r="C53" s="15"/>
@@ -3888,7 +4028,7 @@
       <c r="G53" s="16"/>
       <c r="H53" s="14"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="16"/>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
@@ -3898,7 +4038,7 @@
       <c r="G54" s="16"/>
       <c r="H54" s="14"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="16"/>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
@@ -3908,7 +4048,7 @@
       <c r="G55" s="16"/>
       <c r="H55" s="14"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="16"/>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
@@ -3918,7 +4058,7 @@
       <c r="G56" s="16"/>
       <c r="H56" s="14"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="16"/>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -3928,7 +4068,7 @@
       <c r="G57" s="16"/>
       <c r="H57" s="14"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="16"/>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
@@ -3938,7 +4078,7 @@
       <c r="G58" s="16"/>
       <c r="H58" s="14"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="16"/>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
@@ -3948,7 +4088,7 @@
       <c r="G59" s="16"/>
       <c r="H59" s="14"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="16"/>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
@@ -3958,7 +4098,7 @@
       <c r="G60" s="16"/>
       <c r="H60" s="14"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="16"/>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
@@ -3968,7 +4108,7 @@
       <c r="G61" s="16"/>
       <c r="H61" s="14"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="16"/>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
@@ -3978,7 +4118,7 @@
       <c r="G62" s="16"/>
       <c r="H62" s="14"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="16"/>
       <c r="B63" s="15"/>
       <c r="C63" s="15"/>
@@ -3988,7 +4128,7 @@
       <c r="G63" s="16"/>
       <c r="H63" s="14"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="16"/>
       <c r="B64" s="15"/>
       <c r="C64" s="15"/>
@@ -3998,7 +4138,7 @@
       <c r="G64" s="16"/>
       <c r="H64" s="14"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="16"/>
       <c r="B65" s="15"/>
       <c r="C65" s="15"/>
@@ -4008,7 +4148,7 @@
       <c r="G65" s="16"/>
       <c r="H65" s="14"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="16"/>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
@@ -4018,7 +4158,7 @@
       <c r="G66" s="16"/>
       <c r="H66" s="14"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="16"/>
       <c r="B67" s="15"/>
       <c r="C67" s="15"/>
@@ -4028,7 +4168,7 @@
       <c r="G67" s="16"/>
       <c r="H67" s="14"/>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="16"/>
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
@@ -4038,7 +4178,7 @@
       <c r="G68" s="16"/>
       <c r="H68" s="14"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="16"/>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
@@ -4048,7 +4188,7 @@
       <c r="G69" s="16"/>
       <c r="H69" s="14"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="16"/>
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
@@ -4058,7 +4198,7 @@
       <c r="G70" s="16"/>
       <c r="H70" s="14"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="16"/>
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
@@ -4068,7 +4208,7 @@
       <c r="G71" s="16"/>
       <c r="H71" s="14"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="16"/>
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
@@ -4078,7 +4218,7 @@
       <c r="G72" s="16"/>
       <c r="H72" s="14"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="16"/>
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
@@ -4088,7 +4228,7 @@
       <c r="G73" s="16"/>
       <c r="H73" s="14"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="16"/>
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
@@ -4098,7 +4238,7 @@
       <c r="G74" s="16"/>
       <c r="H74" s="14"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="16"/>
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
@@ -4108,7 +4248,7 @@
       <c r="G75" s="16"/>
       <c r="H75" s="14"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="16"/>
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
@@ -4118,7 +4258,7 @@
       <c r="G76" s="16"/>
       <c r="H76" s="14"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="16"/>
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
@@ -4128,7 +4268,7 @@
       <c r="G77" s="16"/>
       <c r="H77" s="14"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="16"/>
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
@@ -4138,7 +4278,7 @@
       <c r="G78" s="16"/>
       <c r="H78" s="14"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="16"/>
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
@@ -4148,7 +4288,7 @@
       <c r="G79" s="16"/>
       <c r="H79" s="14"/>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="16"/>
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
@@ -4158,7 +4298,7 @@
       <c r="G80" s="16"/>
       <c r="H80" s="14"/>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="16"/>
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
@@ -4168,7 +4308,7 @@
       <c r="G81" s="16"/>
       <c r="H81" s="14"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="16"/>
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
@@ -4178,7 +4318,7 @@
       <c r="G82" s="16"/>
       <c r="H82" s="14"/>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="16"/>
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
@@ -4188,7 +4328,7 @@
       <c r="G83" s="16"/>
       <c r="H83" s="14"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="16"/>
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
@@ -4198,7 +4338,7 @@
       <c r="G84" s="16"/>
       <c r="H84" s="14"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="16"/>
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
@@ -4208,7 +4348,7 @@
       <c r="G85" s="16"/>
       <c r="H85" s="14"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="16"/>
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
@@ -4218,7 +4358,7 @@
       <c r="G86" s="16"/>
       <c r="H86" s="14"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="16"/>
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
@@ -4228,7 +4368,7 @@
       <c r="G87" s="16"/>
       <c r="H87" s="14"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="16"/>
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
@@ -4238,7 +4378,7 @@
       <c r="G88" s="16"/>
       <c r="H88" s="14"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="16"/>
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
@@ -4248,7 +4388,7 @@
       <c r="G89" s="16"/>
       <c r="H89" s="14"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="16"/>
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
@@ -4258,7 +4398,7 @@
       <c r="G90" s="16"/>
       <c r="H90" s="14"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="16"/>
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
@@ -4268,7 +4408,7 @@
       <c r="G91" s="16"/>
       <c r="H91" s="14"/>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="16"/>
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
@@ -4278,7 +4418,7 @@
       <c r="G92" s="16"/>
       <c r="H92" s="14"/>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="16"/>
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
@@ -4288,7 +4428,7 @@
       <c r="G93" s="16"/>
       <c r="H93" s="14"/>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="16"/>
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
@@ -4298,7 +4438,7 @@
       <c r="G94" s="16"/>
       <c r="H94" s="14"/>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="16"/>
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
@@ -4308,7 +4448,7 @@
       <c r="G95" s="16"/>
       <c r="H95" s="14"/>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="16"/>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
@@ -4318,7 +4458,7 @@
       <c r="G96" s="16"/>
       <c r="H96" s="14"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="16"/>
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
@@ -4328,7 +4468,7 @@
       <c r="G97" s="16"/>
       <c r="H97" s="14"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="16"/>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
@@ -4338,7 +4478,7 @@
       <c r="G98" s="16"/>
       <c r="H98" s="14"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="16"/>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
@@ -4348,7 +4488,7 @@
       <c r="G99" s="16"/>
       <c r="H99" s="14"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="16"/>
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
@@ -4358,7 +4498,7 @@
       <c r="G100" s="16"/>
       <c r="H100" s="14"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="16"/>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
@@ -4368,7 +4508,7 @@
       <c r="G101" s="16"/>
       <c r="H101" s="14"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="16"/>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
@@ -4378,7 +4518,7 @@
       <c r="G102" s="16"/>
       <c r="H102" s="14"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="16"/>
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
@@ -4388,7 +4528,7 @@
       <c r="G103" s="16"/>
       <c r="H103" s="14"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="16"/>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
@@ -4398,7 +4538,7 @@
       <c r="G104" s="16"/>
       <c r="H104" s="14"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="16"/>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
@@ -4408,7 +4548,7 @@
       <c r="G105" s="16"/>
       <c r="H105" s="14"/>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="16"/>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
@@ -4418,7 +4558,7 @@
       <c r="G106" s="16"/>
       <c r="H106" s="14"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="16"/>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
@@ -4428,7 +4568,7 @@
       <c r="G107" s="16"/>
       <c r="H107" s="14"/>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="16"/>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
@@ -4438,7 +4578,7 @@
       <c r="G108" s="16"/>
       <c r="H108" s="14"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="16"/>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
@@ -4448,7 +4588,7 @@
       <c r="G109" s="16"/>
       <c r="H109" s="14"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="16"/>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
@@ -4458,7 +4598,7 @@
       <c r="G110" s="16"/>
       <c r="H110" s="14"/>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="16"/>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
@@ -4468,7 +4608,7 @@
       <c r="G111" s="16"/>
       <c r="H111" s="14"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="38"/>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
@@ -4478,7 +4618,7 @@
       <c r="G112" s="16"/>
       <c r="H112" s="14"/>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="50"/>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
@@ -4488,7 +4628,7 @@
       <c r="G113" s="16"/>
       <c r="H113" s="14"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="16"/>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
@@ -4498,7 +4638,7 @@
       <c r="G114" s="56"/>
       <c r="H114" s="14"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="16"/>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
@@ -4508,7 +4648,7 @@
       <c r="G115" s="56"/>
       <c r="H115" s="14"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="38"/>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
@@ -4518,7 +4658,7 @@
       <c r="G116" s="56"/>
       <c r="H116" s="14"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="50"/>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
@@ -4528,7 +4668,7 @@
       <c r="G117" s="56"/>
       <c r="H117" s="14"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="16"/>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -4538,7 +4678,7 @@
       <c r="G118" s="56"/>
       <c r="H118" s="14"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="16"/>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
@@ -4548,7 +4688,7 @@
       <c r="G119" s="56"/>
       <c r="H119" s="14"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="38"/>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
@@ -4558,7 +4698,7 @@
       <c r="G120" s="56"/>
       <c r="H120" s="14"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="50"/>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
@@ -4568,7 +4708,7 @@
       <c r="G121" s="56"/>
       <c r="H121" s="14"/>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="16"/>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
@@ -4578,7 +4718,7 @@
       <c r="G122" s="56"/>
       <c r="H122" s="14"/>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="16"/>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
@@ -4588,7 +4728,7 @@
       <c r="G123" s="56"/>
       <c r="H123" s="14"/>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" s="38"/>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
@@ -4598,7 +4738,7 @@
       <c r="G124" s="56"/>
       <c r="H124" s="14"/>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="50"/>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
@@ -4608,7 +4748,7 @@
       <c r="G125" s="56"/>
       <c r="H125" s="14"/>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="16"/>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
@@ -4618,7 +4758,7 @@
       <c r="G126" s="56"/>
       <c r="H126" s="14"/>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="16"/>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
@@ -4628,7 +4768,7 @@
       <c r="G127" s="56"/>
       <c r="H127" s="14"/>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="38"/>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
@@ -4638,7 +4778,7 @@
       <c r="G128" s="56"/>
       <c r="H128" s="14"/>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="50"/>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
@@ -4648,7 +4788,7 @@
       <c r="G129" s="56"/>
       <c r="H129" s="14"/>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" s="16"/>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
@@ -4658,7 +4798,7 @@
       <c r="G130" s="56"/>
       <c r="H130" s="14"/>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="16"/>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
@@ -4668,7 +4808,7 @@
       <c r="G131" s="56"/>
       <c r="H131" s="14"/>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="38"/>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
@@ -4678,7 +4818,7 @@
       <c r="G132" s="56"/>
       <c r="H132" s="14"/>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="50"/>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
@@ -4688,7 +4828,7 @@
       <c r="G133" s="56"/>
       <c r="H133" s="14"/>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="16"/>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
@@ -4698,7 +4838,7 @@
       <c r="G134" s="56"/>
       <c r="H134" s="14"/>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="16"/>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
@@ -4708,7 +4848,7 @@
       <c r="G135" s="56"/>
       <c r="H135" s="14"/>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" s="38"/>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
@@ -4718,7 +4858,7 @@
       <c r="G136" s="56"/>
       <c r="H136" s="14"/>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" s="50"/>
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
@@ -4728,7 +4868,7 @@
       <c r="G137" s="56"/>
       <c r="H137" s="14"/>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" s="16"/>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
@@ -4738,7 +4878,7 @@
       <c r="G138" s="56"/>
       <c r="H138" s="14"/>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="16"/>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
@@ -4748,7 +4888,7 @@
       <c r="G139" s="56"/>
       <c r="H139" s="14"/>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" s="38"/>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
@@ -4758,7 +4898,7 @@
       <c r="G140" s="56"/>
       <c r="H140" s="14"/>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" s="50"/>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
@@ -4768,7 +4908,7 @@
       <c r="G141" s="56"/>
       <c r="H141" s="14"/>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" s="16"/>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
@@ -4778,7 +4918,7 @@
       <c r="G142" s="56"/>
       <c r="H142" s="14"/>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="16"/>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
@@ -4788,7 +4928,7 @@
       <c r="G143" s="56"/>
       <c r="H143" s="14"/>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" s="38"/>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
@@ -4798,7 +4938,7 @@
       <c r="G144" s="56"/>
       <c r="H144" s="14"/>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" s="50"/>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
@@ -4808,7 +4948,7 @@
       <c r="G145" s="56"/>
       <c r="H145" s="14"/>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="16"/>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
@@ -4818,7 +4958,7 @@
       <c r="G146" s="56"/>
       <c r="H146" s="14"/>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="16"/>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
@@ -4828,7 +4968,7 @@
       <c r="G147" s="56"/>
       <c r="H147" s="14"/>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="38"/>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
@@ -4838,7 +4978,7 @@
       <c r="G148" s="56"/>
       <c r="H148" s="14"/>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" s="50"/>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
@@ -4848,7 +4988,7 @@
       <c r="G149" s="56"/>
       <c r="H149" s="14"/>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" s="16"/>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
@@ -4858,7 +4998,7 @@
       <c r="G150" s="56"/>
       <c r="H150" s="14"/>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" s="16"/>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
@@ -4868,7 +5008,7 @@
       <c r="G151" s="56"/>
       <c r="H151" s="14"/>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" s="38"/>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
@@ -4878,7 +5018,7 @@
       <c r="G152" s="56"/>
       <c r="H152" s="14"/>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A153" s="50"/>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
@@ -4888,7 +5028,7 @@
       <c r="G153" s="56"/>
       <c r="H153" s="14"/>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A154" s="16"/>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
@@ -4898,7 +5038,7 @@
       <c r="G154" s="56"/>
       <c r="H154" s="14"/>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155" s="16"/>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
@@ -4908,7 +5048,7 @@
       <c r="G155" s="56"/>
       <c r="H155" s="14"/>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" s="38"/>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
@@ -4918,7 +5058,7 @@
       <c r="G156" s="56"/>
       <c r="H156" s="14"/>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A157" s="50"/>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
@@ -4928,7 +5068,7 @@
       <c r="G157" s="56"/>
       <c r="H157" s="14"/>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A158" s="16"/>
       <c r="B158" s="15"/>
       <c r="C158" s="15"/>
@@ -4938,7 +5078,7 @@
       <c r="G158" s="56"/>
       <c r="H158" s="14"/>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A159" s="16"/>
       <c r="B159" s="15"/>
       <c r="C159" s="15"/>
@@ -4948,7 +5088,7 @@
       <c r="G159" s="56"/>
       <c r="H159" s="14"/>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A160" s="38"/>
       <c r="B160" s="15"/>
       <c r="C160" s="15"/>
@@ -4958,7 +5098,7 @@
       <c r="G160" s="56"/>
       <c r="H160" s="14"/>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A161" s="50"/>
       <c r="B161" s="15"/>
       <c r="C161" s="15"/>
@@ -4968,7 +5108,7 @@
       <c r="G161" s="56"/>
       <c r="H161" s="14"/>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A162" s="16"/>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
@@ -4978,7 +5118,7 @@
       <c r="G162" s="56"/>
       <c r="H162" s="14"/>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A163" s="16"/>
       <c r="B163" s="15"/>
       <c r="C163" s="15"/>
@@ -4988,7 +5128,7 @@
       <c r="G163" s="56"/>
       <c r="H163" s="14"/>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A164" s="38"/>
       <c r="B164" s="15"/>
       <c r="C164" s="15"/>
@@ -4998,7 +5138,7 @@
       <c r="G164" s="56"/>
       <c r="H164" s="14"/>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" s="50"/>
       <c r="B165" s="15"/>
       <c r="C165" s="15"/>
@@ -5008,7 +5148,7 @@
       <c r="G165" s="56"/>
       <c r="H165" s="14"/>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A166" s="16"/>
       <c r="B166" s="15"/>
       <c r="C166" s="15"/>
@@ -5018,7 +5158,7 @@
       <c r="G166" s="56"/>
       <c r="H166" s="14"/>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A167" s="16"/>
       <c r="B167" s="15"/>
       <c r="C167" s="15"/>
@@ -5028,7 +5168,7 @@
       <c r="G167" s="56"/>
       <c r="H167" s="14"/>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A168" s="38"/>
       <c r="B168" s="15"/>
       <c r="C168" s="15"/>
@@ -5038,7 +5178,7 @@
       <c r="G168" s="56"/>
       <c r="H168" s="14"/>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A169" s="50"/>
       <c r="B169" s="15"/>
       <c r="C169" s="15"/>
@@ -5048,7 +5188,7 @@
       <c r="G169" s="56"/>
       <c r="H169" s="14"/>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A170" s="16"/>
       <c r="B170" s="15"/>
       <c r="C170" s="15"/>
@@ -5058,7 +5198,7 @@
       <c r="G170" s="56"/>
       <c r="H170" s="14"/>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A171" s="16"/>
       <c r="B171" s="15"/>
       <c r="C171" s="15"/>
@@ -5068,7 +5208,7 @@
       <c r="G171" s="56"/>
       <c r="H171" s="14"/>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A172" s="38"/>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -5078,7 +5218,7 @@
       <c r="G172" s="56"/>
       <c r="H172" s="14"/>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A173" s="50"/>
       <c r="B173" s="15"/>
       <c r="C173" s="15"/>
@@ -5088,7 +5228,7 @@
       <c r="G173" s="56"/>
       <c r="H173" s="14"/>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A174" s="16"/>
       <c r="B174" s="15"/>
       <c r="C174" s="15"/>
@@ -5098,7 +5238,7 @@
       <c r="G174" s="56"/>
       <c r="H174" s="14"/>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A175" s="16"/>
       <c r="B175" s="15"/>
       <c r="C175" s="15"/>
@@ -5108,7 +5248,7 @@
       <c r="G175" s="56"/>
       <c r="H175" s="14"/>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A176" s="38"/>
       <c r="B176" s="15"/>
       <c r="C176" s="15"/>
@@ -5118,7 +5258,7 @@
       <c r="G176" s="56"/>
       <c r="H176" s="14"/>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A177" s="50"/>
       <c r="B177" s="15"/>
       <c r="C177" s="15"/>
@@ -5128,7 +5268,7 @@
       <c r="G177" s="56"/>
       <c r="H177" s="14"/>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A178" s="16"/>
       <c r="B178" s="15"/>
       <c r="C178" s="15"/>
@@ -5138,7 +5278,7 @@
       <c r="G178" s="56"/>
       <c r="H178" s="14"/>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A179" s="16"/>
       <c r="B179" s="15"/>
       <c r="C179" s="15"/>
@@ -5148,7 +5288,7 @@
       <c r="G179" s="56"/>
       <c r="H179" s="14"/>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A180" s="38"/>
       <c r="B180" s="15"/>
       <c r="C180" s="15"/>
@@ -5158,7 +5298,7 @@
       <c r="G180" s="56"/>
       <c r="H180" s="14"/>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A181" s="50"/>
       <c r="B181" s="15"/>
       <c r="C181" s="15"/>
@@ -5168,7 +5308,7 @@
       <c r="G181" s="56"/>
       <c r="H181" s="14"/>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A182" s="16"/>
       <c r="B182" s="15"/>
       <c r="C182" s="15"/>
@@ -5178,7 +5318,7 @@
       <c r="G182" s="56"/>
       <c r="H182" s="14"/>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A183" s="16"/>
       <c r="B183" s="15"/>
       <c r="C183" s="15"/>
@@ -5188,7 +5328,7 @@
       <c r="G183" s="56"/>
       <c r="H183" s="14"/>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A184" s="38"/>
       <c r="B184" s="15"/>
       <c r="C184" s="15"/>
@@ -5198,7 +5338,7 @@
       <c r="G184" s="56"/>
       <c r="H184" s="14"/>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A185" s="50"/>
       <c r="B185" s="15"/>
       <c r="C185" s="15"/>
@@ -5208,7 +5348,7 @@
       <c r="G185" s="56"/>
       <c r="H185" s="14"/>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A186" s="16"/>
       <c r="B186" s="15"/>
       <c r="C186" s="15"/>
@@ -5218,7 +5358,7 @@
       <c r="G186" s="56"/>
       <c r="H186" s="14"/>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A187" s="16"/>
       <c r="B187" s="15"/>
       <c r="C187" s="15"/>
@@ -5228,7 +5368,7 @@
       <c r="G187" s="56"/>
       <c r="H187" s="14"/>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A188" s="38"/>
       <c r="B188" s="15"/>
       <c r="C188" s="15"/>
@@ -5238,7 +5378,7 @@
       <c r="G188" s="56"/>
       <c r="H188" s="14"/>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A189" s="50"/>
       <c r="B189" s="15"/>
       <c r="C189" s="15"/>
@@ -5248,7 +5388,7 @@
       <c r="G189" s="56"/>
       <c r="H189" s="14"/>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A190" s="16"/>
       <c r="B190" s="15"/>
       <c r="C190" s="15"/>
@@ -5258,7 +5398,7 @@
       <c r="G190" s="56"/>
       <c r="H190" s="14"/>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A191" s="16"/>
       <c r="B191" s="15"/>
       <c r="C191" s="15"/>
@@ -5268,7 +5408,7 @@
       <c r="G191" s="56"/>
       <c r="H191" s="14"/>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A192" s="38"/>
       <c r="B192" s="15"/>
       <c r="C192" s="15"/>
@@ -5278,7 +5418,7 @@
       <c r="G192" s="56"/>
       <c r="H192" s="14"/>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A193" s="50"/>
       <c r="B193" s="15"/>
       <c r="C193" s="15"/>
@@ -5288,7 +5428,7 @@
       <c r="G193" s="56"/>
       <c r="H193" s="14"/>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A194" s="16"/>
       <c r="B194" s="15"/>
       <c r="C194" s="15"/>
@@ -5298,7 +5438,7 @@
       <c r="G194" s="56"/>
       <c r="H194" s="14"/>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A195" s="16"/>
       <c r="B195" s="15"/>
       <c r="C195" s="15"/>
@@ -5308,7 +5448,7 @@
       <c r="G195" s="56"/>
       <c r="H195" s="14"/>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A196" s="38"/>
       <c r="B196" s="15"/>
       <c r="C196" s="15"/>
@@ -5318,7 +5458,7 @@
       <c r="G196" s="56"/>
       <c r="H196" s="14"/>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" s="50"/>
       <c r="B197" s="15"/>
       <c r="C197" s="15"/>
@@ -5328,7 +5468,7 @@
       <c r="G197" s="56"/>
       <c r="H197" s="14"/>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A198" s="16"/>
       <c r="B198" s="15"/>
       <c r="C198" s="15"/>
@@ -5338,7 +5478,7 @@
       <c r="G198" s="56"/>
       <c r="H198" s="14"/>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A199" s="16"/>
       <c r="B199" s="15"/>
       <c r="C199" s="15"/>
@@ -5348,7 +5488,7 @@
       <c r="G199" s="56"/>
       <c r="H199" s="14"/>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A200" s="38"/>
       <c r="B200" s="15"/>
       <c r="C200" s="15"/>
@@ -5358,7 +5498,7 @@
       <c r="G200" s="56"/>
       <c r="H200" s="14"/>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A201" s="50"/>
       <c r="B201" s="15"/>
       <c r="C201" s="15"/>
@@ -5368,7 +5508,7 @@
       <c r="G201" s="56"/>
       <c r="H201" s="14"/>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A202" s="16"/>
       <c r="B202" s="15"/>
       <c r="C202" s="15"/>
@@ -5378,7 +5518,7 @@
       <c r="G202" s="56"/>
       <c r="H202" s="14"/>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A203" s="16"/>
       <c r="B203" s="15"/>
       <c r="C203" s="15"/>
@@ -5388,7 +5528,7 @@
       <c r="G203" s="56"/>
       <c r="H203" s="14"/>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A204" s="38"/>
       <c r="B204" s="15"/>
       <c r="C204" s="15"/>
@@ -5398,7 +5538,7 @@
       <c r="G204" s="56"/>
       <c r="H204" s="14"/>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A205" s="50"/>
       <c r="B205" s="15"/>
       <c r="C205" s="15"/>
@@ -5408,7 +5548,7 @@
       <c r="G205" s="56"/>
       <c r="H205" s="14"/>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A206" s="16"/>
       <c r="B206" s="15"/>
       <c r="C206" s="15"/>
@@ -5418,7 +5558,7 @@
       <c r="G206" s="56"/>
       <c r="H206" s="14"/>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A207" s="16"/>
       <c r="B207" s="15"/>
       <c r="C207" s="15"/>
@@ -5428,7 +5568,7 @@
       <c r="G207" s="56"/>
       <c r="H207" s="14"/>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A208" s="38"/>
       <c r="B208" s="15"/>
       <c r="C208" s="15"/>
@@ -5438,7 +5578,7 @@
       <c r="G208" s="56"/>
       <c r="H208" s="14"/>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A209" s="50"/>
       <c r="B209" s="15"/>
       <c r="C209" s="15"/>
@@ -5448,7 +5588,7 @@
       <c r="G209" s="56"/>
       <c r="H209" s="14"/>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A210" s="16"/>
       <c r="B210" s="15"/>
       <c r="C210" s="15"/>
@@ -5458,7 +5598,7 @@
       <c r="G210" s="56"/>
       <c r="H210" s="14"/>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A211" s="16"/>
       <c r="B211" s="15"/>
       <c r="C211" s="15"/>
@@ -5468,7 +5608,7 @@
       <c r="G211" s="56"/>
       <c r="H211" s="14"/>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A212" s="38"/>
       <c r="B212" s="15"/>
       <c r="C212" s="15"/>
@@ -5478,7 +5618,7 @@
       <c r="G212" s="56"/>
       <c r="H212" s="14"/>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A213" s="50"/>
       <c r="B213" s="15"/>
       <c r="C213" s="15"/>
@@ -5488,7 +5628,7 @@
       <c r="G213" s="56"/>
       <c r="H213" s="14"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A214" s="16"/>
       <c r="B214" s="15"/>
       <c r="C214" s="15"/>
@@ -5498,7 +5638,7 @@
       <c r="G214" s="56"/>
       <c r="H214" s="14"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A215" s="16"/>
       <c r="B215" s="15"/>
       <c r="C215" s="15"/>
@@ -5508,7 +5648,7 @@
       <c r="G215" s="56"/>
       <c r="H215" s="14"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A216" s="38"/>
       <c r="B216" s="15"/>
       <c r="C216" s="15"/>
@@ -5518,7 +5658,7 @@
       <c r="G216" s="56"/>
       <c r="H216" s="14"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A217" s="50"/>
       <c r="B217" s="15"/>
       <c r="C217" s="15"/>
@@ -5528,7 +5668,7 @@
       <c r="G217" s="56"/>
       <c r="H217" s="14"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A218" s="16"/>
       <c r="B218" s="15"/>
       <c r="C218" s="15"/>
@@ -5538,7 +5678,7 @@
       <c r="G218" s="56"/>
       <c r="H218" s="14"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A219" s="16"/>
       <c r="B219" s="15"/>
       <c r="C219" s="15"/>
@@ -5548,7 +5688,7 @@
       <c r="G219" s="56"/>
       <c r="H219" s="14"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A220" s="38"/>
       <c r="B220" s="15"/>
       <c r="C220" s="15"/>
@@ -5558,7 +5698,7 @@
       <c r="G220" s="56"/>
       <c r="H220" s="14"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A221" s="50"/>
       <c r="B221" s="15"/>
       <c r="C221" s="15"/>
@@ -5568,7 +5708,7 @@
       <c r="G221" s="56"/>
       <c r="H221" s="14"/>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A222" s="16"/>
       <c r="B222" s="15"/>
       <c r="C222" s="15"/>
@@ -5578,7 +5718,7 @@
       <c r="G222" s="56"/>
       <c r="H222" s="14"/>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A223" s="16"/>
       <c r="B223" s="15"/>
       <c r="C223" s="15"/>
@@ -5588,7 +5728,7 @@
       <c r="G223" s="56"/>
       <c r="H223" s="14"/>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A224" s="38"/>
       <c r="B224" s="15"/>
       <c r="C224" s="15"/>
@@ -5598,7 +5738,7 @@
       <c r="G224" s="56"/>
       <c r="H224" s="14"/>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A225" s="50"/>
       <c r="B225" s="15"/>
       <c r="C225" s="15"/>
@@ -5608,7 +5748,7 @@
       <c r="G225" s="56"/>
       <c r="H225" s="14"/>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A226" s="16"/>
       <c r="B226" s="15"/>
       <c r="C226" s="15"/>
@@ -5618,7 +5758,7 @@
       <c r="G226" s="56"/>
       <c r="H226" s="14"/>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A227" s="16"/>
       <c r="B227" s="15"/>
       <c r="C227" s="15"/>
@@ -5628,7 +5768,7 @@
       <c r="G227" s="56"/>
       <c r="H227" s="14"/>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A228" s="38"/>
       <c r="B228" s="15"/>
       <c r="C228" s="15"/>
@@ -5638,7 +5778,7 @@
       <c r="G228" s="56"/>
       <c r="H228" s="14"/>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A229" s="50"/>
       <c r="B229" s="15"/>
       <c r="C229" s="15"/>
@@ -5648,7 +5788,7 @@
       <c r="G229" s="56"/>
       <c r="H229" s="14"/>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A230" s="16"/>
       <c r="B230" s="15"/>
       <c r="C230" s="15"/>
@@ -5658,7 +5798,7 @@
       <c r="G230" s="56"/>
       <c r="H230" s="14"/>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A231" s="16"/>
       <c r="B231" s="15"/>
       <c r="C231" s="15"/>
@@ -5666,7 +5806,7 @@
       <c r="G231" s="56"/>
       <c r="H231" s="14"/>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A232" s="16"/>
       <c r="B232" s="15"/>
       <c r="C232" s="15"/>
@@ -5674,7 +5814,7 @@
       <c r="G232" s="56"/>
       <c r="H232" s="14"/>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A233" s="38"/>
       <c r="B233" s="15"/>
       <c r="C233" s="15"/>
@@ -5682,7 +5822,7 @@
       <c r="G233" s="56"/>
       <c r="H233" s="14"/>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A234" s="50"/>
       <c r="B234" s="15"/>
       <c r="C234" s="15"/>
@@ -5690,7 +5830,7 @@
       <c r="G234" s="56"/>
       <c r="H234" s="14"/>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A235" s="16"/>
       <c r="B235" s="15"/>
       <c r="C235" s="15"/>
@@ -5698,7 +5838,7 @@
       <c r="G235" s="56"/>
       <c r="H235" s="14"/>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A236" s="16"/>
       <c r="B236" s="15"/>
       <c r="C236" s="15"/>
@@ -5706,7 +5846,7 @@
       <c r="G236" s="56"/>
       <c r="H236" s="14"/>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A237" s="16"/>
       <c r="B237" s="15"/>
       <c r="C237" s="15"/>
@@ -5714,7 +5854,7 @@
       <c r="G237" s="56"/>
       <c r="H237" s="14"/>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A238" s="38"/>
       <c r="B238" s="15"/>
       <c r="C238" s="15"/>
@@ -5722,7 +5862,7 @@
       <c r="G238" s="56"/>
       <c r="H238" s="14"/>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A239" s="50"/>
       <c r="B239" s="15"/>
       <c r="C239" s="15"/>
@@ -5730,7 +5870,7 @@
       <c r="G239" s="56"/>
       <c r="H239" s="14"/>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A240" s="16"/>
       <c r="B240" s="15"/>
       <c r="C240" s="15"/>
@@ -5738,7 +5878,7 @@
       <c r="G240" s="56"/>
       <c r="H240" s="14"/>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A241" s="16"/>
       <c r="B241" s="15"/>
       <c r="C241" s="15"/>
@@ -5746,7 +5886,7 @@
       <c r="G241" s="56"/>
       <c r="H241" s="14"/>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A242" s="16"/>
       <c r="B242" s="15"/>
       <c r="C242" s="15"/>
@@ -5754,7 +5894,7 @@
       <c r="G242" s="56"/>
       <c r="H242" s="14"/>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A243" s="38"/>
       <c r="B243" s="15"/>
       <c r="C243" s="15"/>
@@ -5762,7 +5902,7 @@
       <c r="G243" s="56"/>
       <c r="H243" s="14"/>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A244" s="50"/>
       <c r="B244" s="15"/>
       <c r="C244" s="15"/>
@@ -5770,7 +5910,7 @@
       <c r="G244" s="56"/>
       <c r="H244" s="14"/>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A245" s="16"/>
       <c r="B245" s="15"/>
       <c r="C245" s="15"/>
@@ -5778,7 +5918,7 @@
       <c r="G245" s="56"/>
       <c r="H245" s="14"/>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A246" s="16"/>
       <c r="B246" s="15"/>
       <c r="C246" s="15"/>
@@ -5786,7 +5926,7 @@
       <c r="G246" s="56"/>
       <c r="H246" s="14"/>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A247" s="16"/>
       <c r="B247" s="15"/>
       <c r="C247" s="15"/>
@@ -5794,7 +5934,7 @@
       <c r="G247" s="56"/>
       <c r="H247" s="14"/>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A248" s="38"/>
       <c r="B248" s="15"/>
       <c r="C248" s="15"/>
@@ -5802,7 +5942,7 @@
       <c r="G248" s="56"/>
       <c r="H248" s="14"/>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A249" s="50"/>
       <c r="B249" s="15"/>
       <c r="C249" s="15"/>
@@ -5810,7 +5950,7 @@
       <c r="G249" s="56"/>
       <c r="H249" s="14"/>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A250" s="16"/>
       <c r="B250" s="15"/>
       <c r="C250" s="15"/>
@@ -5818,7 +5958,7 @@
       <c r="G250" s="56"/>
       <c r="H250" s="14"/>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A251" s="16"/>
       <c r="B251" s="15"/>
       <c r="C251" s="15"/>
@@ -5826,7 +5966,7 @@
       <c r="G251" s="56"/>
       <c r="H251" s="14"/>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A252" s="16"/>
       <c r="B252" s="15"/>
       <c r="C252" s="15"/>
@@ -5834,7 +5974,7 @@
       <c r="G252" s="56"/>
       <c r="H252" s="14"/>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A253" s="38"/>
       <c r="B253" s="15"/>
       <c r="C253" s="15"/>
@@ -5842,7 +5982,7 @@
       <c r="G253" s="56"/>
       <c r="H253" s="14"/>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A254" s="50"/>
       <c r="B254" s="15"/>
       <c r="C254" s="15"/>
@@ -5850,7 +5990,7 @@
       <c r="G254" s="56"/>
       <c r="H254" s="14"/>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A255" s="16"/>
       <c r="B255" s="15"/>
       <c r="C255" s="15"/>
@@ -5858,7 +5998,7 @@
       <c r="G255" s="56"/>
       <c r="H255" s="14"/>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A256" s="16"/>
       <c r="B256" s="15"/>
       <c r="C256" s="15"/>
@@ -5866,7 +6006,7 @@
       <c r="G256" s="56"/>
       <c r="H256" s="14"/>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A257" s="16"/>
       <c r="B257" s="15"/>
       <c r="C257" s="15"/>
@@ -5874,7 +6014,7 @@
       <c r="G257" s="56"/>
       <c r="H257" s="14"/>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A258" s="38"/>
       <c r="B258" s="15"/>
       <c r="C258" s="15"/>
@@ -5882,7 +6022,7 @@
       <c r="G258" s="56"/>
       <c r="H258" s="14"/>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A259" s="50"/>
       <c r="B259" s="15"/>
       <c r="C259" s="15"/>
@@ -5890,7 +6030,7 @@
       <c r="G259" s="56"/>
       <c r="H259" s="14"/>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A260" s="16"/>
       <c r="B260" s="15"/>
       <c r="C260" s="15"/>
@@ -5898,7 +6038,7 @@
       <c r="G260" s="56"/>
       <c r="H260" s="14"/>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A261" s="16"/>
       <c r="B261" s="15"/>
       <c r="C261" s="15"/>
@@ -5906,7 +6046,7 @@
       <c r="G261" s="56"/>
       <c r="H261" s="14"/>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A262" s="16"/>
       <c r="B262" s="15"/>
       <c r="C262" s="15"/>
@@ -5914,7 +6054,7 @@
       <c r="G262" s="56"/>
       <c r="H262" s="14"/>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A263" s="38"/>
       <c r="B263" s="15"/>
       <c r="C263" s="15"/>
@@ -5922,7 +6062,7 @@
       <c r="G263" s="56"/>
       <c r="H263" s="14"/>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A264" s="50"/>
       <c r="B264" s="15"/>
       <c r="C264" s="15"/>
@@ -5930,7 +6070,7 @@
       <c r="G264" s="56"/>
       <c r="H264" s="14"/>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A265" s="16"/>
       <c r="B265" s="15"/>
       <c r="C265" s="15"/>
@@ -5938,7 +6078,7 @@
       <c r="G265" s="56"/>
       <c r="H265" s="14"/>
     </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A266" s="16"/>
       <c r="B266" s="15"/>
       <c r="C266" s="15"/>
@@ -5946,7 +6086,7 @@
       <c r="G266" s="56"/>
       <c r="H266" s="14"/>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A267" s="16"/>
       <c r="B267" s="15"/>
       <c r="C267" s="15"/>
@@ -5954,7 +6094,7 @@
       <c r="G267" s="56"/>
       <c r="H267" s="14"/>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A268" s="38"/>
       <c r="B268" s="15"/>
       <c r="C268" s="15"/>
@@ -5962,7 +6102,7 @@
       <c r="G268" s="56"/>
       <c r="H268" s="14"/>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A269" s="50"/>
       <c r="B269" s="15"/>
       <c r="C269" s="15"/>
@@ -5970,7 +6110,7 @@
       <c r="G269" s="56"/>
       <c r="H269" s="14"/>
     </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A270" s="16"/>
       <c r="B270" s="15"/>
       <c r="C270" s="15"/>
@@ -5978,7 +6118,7 @@
       <c r="G270" s="56"/>
       <c r="H270" s="14"/>
     </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A271" s="16"/>
       <c r="B271" s="15"/>
       <c r="C271" s="15"/>
@@ -5986,7 +6126,7 @@
       <c r="G271" s="56"/>
       <c r="H271" s="14"/>
     </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A272" s="16"/>
       <c r="B272" s="15"/>
       <c r="C272" s="15"/>
@@ -5994,7 +6134,7 @@
       <c r="G272" s="56"/>
       <c r="H272" s="14"/>
     </row>
-    <row r="273" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A273" s="38"/>
       <c r="B273" s="15"/>
       <c r="C273" s="15"/>
@@ -6002,7 +6142,7 @@
       <c r="G273" s="56"/>
       <c r="H273" s="14"/>
     </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A274" s="50"/>
       <c r="B274" s="15"/>
       <c r="C274" s="15"/>
@@ -6010,7 +6150,7 @@
       <c r="G274" s="56"/>
       <c r="H274" s="14"/>
     </row>
-    <row r="275" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A275" s="16"/>
       <c r="B275" s="15"/>
       <c r="C275" s="15"/>
@@ -6018,7 +6158,7 @@
       <c r="G275" s="56"/>
       <c r="H275" s="14"/>
     </row>
-    <row r="276" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A276" s="16"/>
       <c r="B276" s="15"/>
       <c r="C276" s="15"/>
@@ -6026,7 +6166,7 @@
       <c r="G276" s="56"/>
       <c r="H276" s="14"/>
     </row>
-    <row r="277" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A277" s="16"/>
       <c r="B277" s="15"/>
       <c r="C277" s="15"/>
@@ -6034,7 +6174,7 @@
       <c r="G277" s="56"/>
       <c r="H277" s="14"/>
     </row>
-    <row r="278" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A278" s="38"/>
       <c r="B278" s="15"/>
       <c r="C278" s="15"/>
@@ -6042,7 +6182,7 @@
       <c r="G278" s="56"/>
       <c r="H278" s="14"/>
     </row>
-    <row r="279" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A279" s="50"/>
       <c r="B279" s="15"/>
       <c r="C279" s="15"/>
@@ -6050,7 +6190,7 @@
       <c r="G279" s="56"/>
       <c r="H279" s="14"/>
     </row>
-    <row r="280" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A280" s="16"/>
       <c r="B280" s="15"/>
       <c r="C280" s="15"/>
@@ -6058,7 +6198,7 @@
       <c r="G280" s="56"/>
       <c r="H280" s="14"/>
     </row>
-    <row r="281" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A281" s="16"/>
       <c r="B281" s="15"/>
       <c r="C281" s="15"/>
@@ -6066,7 +6206,7 @@
       <c r="G281" s="56"/>
       <c r="H281" s="14"/>
     </row>
-    <row r="282" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A282" s="16"/>
       <c r="B282" s="15"/>
       <c r="C282" s="15"/>
@@ -6074,7 +6214,7 @@
       <c r="G282" s="56"/>
       <c r="H282" s="14"/>
     </row>
-    <row r="283" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A283" s="38"/>
       <c r="B283" s="15"/>
       <c r="C283" s="15"/>
@@ -6082,7 +6222,7 @@
       <c r="G283" s="56"/>
       <c r="H283" s="14"/>
     </row>
-    <row r="284" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A284" s="50"/>
       <c r="B284" s="15"/>
       <c r="C284" s="15"/>
@@ -6090,7 +6230,7 @@
       <c r="G284" s="56"/>
       <c r="H284" s="14"/>
     </row>
-    <row r="285" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A285" s="16"/>
       <c r="B285" s="15"/>
       <c r="C285" s="15"/>
@@ -6098,7 +6238,7 @@
       <c r="G285" s="56"/>
       <c r="H285" s="14"/>
     </row>
-    <row r="286" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A286" s="16"/>
       <c r="B286" s="15"/>
       <c r="C286" s="15"/>
@@ -6106,7 +6246,7 @@
       <c r="G286" s="56"/>
       <c r="H286" s="14"/>
     </row>
-    <row r="287" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A287" s="16"/>
       <c r="B287" s="15"/>
       <c r="C287" s="15"/>
@@ -6114,7 +6254,7 @@
       <c r="G287" s="56"/>
       <c r="H287" s="14"/>
     </row>
-    <row r="288" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A288" s="38"/>
       <c r="B288" s="15"/>
       <c r="C288" s="15"/>
@@ -6122,7 +6262,7 @@
       <c r="G288" s="56"/>
       <c r="H288" s="14"/>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A289" s="50"/>
       <c r="B289" s="15"/>
       <c r="C289" s="15"/>
@@ -6130,7 +6270,7 @@
       <c r="G289" s="56"/>
       <c r="H289" s="14"/>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A290" s="16"/>
       <c r="B290" s="15"/>
       <c r="C290" s="15"/>
@@ -6138,7 +6278,7 @@
       <c r="G290" s="56"/>
       <c r="H290" s="14"/>
     </row>
-    <row r="291" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A291" s="16"/>
       <c r="B291" s="15"/>
       <c r="C291" s="15"/>
@@ -6146,7 +6286,7 @@
       <c r="G291" s="56"/>
       <c r="H291" s="14"/>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A292" s="16"/>
       <c r="B292" s="15"/>
       <c r="C292" s="15"/>
@@ -6154,7 +6294,7 @@
       <c r="G292" s="56"/>
       <c r="H292" s="14"/>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A293" s="38"/>
       <c r="B293" s="15"/>
       <c r="C293" s="15"/>
@@ -6162,7 +6302,7 @@
       <c r="G293" s="56"/>
       <c r="H293" s="14"/>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A294" s="50"/>
       <c r="B294" s="15"/>
       <c r="C294" s="15"/>
@@ -6170,7 +6310,7 @@
       <c r="G294" s="56"/>
       <c r="H294" s="14"/>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A295" s="16"/>
       <c r="B295" s="15"/>
       <c r="C295" s="15"/>
@@ -6178,7 +6318,7 @@
       <c r="G295" s="56"/>
       <c r="H295" s="14"/>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A296" s="16"/>
       <c r="B296" s="15"/>
       <c r="C296" s="15"/>
@@ -6186,7 +6326,7 @@
       <c r="G296" s="56"/>
       <c r="H296" s="14"/>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A297" s="16"/>
       <c r="B297" s="15"/>
       <c r="C297" s="15"/>
@@ -6194,7 +6334,7 @@
       <c r="G297" s="56"/>
       <c r="H297" s="14"/>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A298" s="38"/>
       <c r="B298" s="15"/>
       <c r="C298" s="15"/>
@@ -6202,7 +6342,7 @@
       <c r="G298" s="56"/>
       <c r="H298" s="14"/>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A299" s="50"/>
       <c r="B299" s="15"/>
       <c r="C299" s="15"/>
@@ -6210,7 +6350,7 @@
       <c r="G299" s="56"/>
       <c r="H299" s="14"/>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A300" s="16"/>
       <c r="B300" s="15"/>
       <c r="C300" s="15"/>
@@ -6218,7 +6358,7 @@
       <c r="G300" s="56"/>
       <c r="H300" s="14"/>
     </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A301" s="16"/>
       <c r="B301" s="15"/>
       <c r="C301" s="15"/>
@@ -6226,7 +6366,7 @@
       <c r="G301" s="56"/>
       <c r="H301" s="14"/>
     </row>
-    <row r="302" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A302" s="16"/>
       <c r="B302" s="15"/>
       <c r="C302" s="15"/>
@@ -6234,7 +6374,7 @@
       <c r="G302" s="56"/>
       <c r="H302" s="14"/>
     </row>
-    <row r="303" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A303" s="38"/>
       <c r="B303" s="15"/>
       <c r="C303" s="15"/>
@@ -6242,7 +6382,7 @@
       <c r="G303" s="56"/>
       <c r="H303" s="14"/>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A304" s="50"/>
       <c r="B304" s="15"/>
       <c r="C304" s="15"/>
@@ -6250,7 +6390,7 @@
       <c r="G304" s="56"/>
       <c r="H304" s="14"/>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A305" s="16"/>
       <c r="B305" s="15"/>
       <c r="C305" s="15"/>
@@ -6258,7 +6398,7 @@
       <c r="G305" s="56"/>
       <c r="H305" s="14"/>
     </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A306" s="16"/>
       <c r="B306" s="15"/>
       <c r="C306" s="15"/>
@@ -6266,7 +6406,7 @@
       <c r="G306" s="56"/>
       <c r="H306" s="14"/>
     </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A307" s="16"/>
       <c r="B307" s="15"/>
       <c r="C307" s="15"/>
@@ -6274,7 +6414,7 @@
       <c r="G307" s="56"/>
       <c r="H307" s="14"/>
     </row>
-    <row r="308" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A308" s="38"/>
       <c r="B308" s="15"/>
       <c r="C308" s="15"/>
@@ -6282,7 +6422,7 @@
       <c r="G308" s="56"/>
       <c r="H308" s="14"/>
     </row>
-    <row r="309" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A309" s="50"/>
       <c r="B309" s="15"/>
       <c r="C309" s="15"/>
@@ -6290,7 +6430,7 @@
       <c r="G309" s="56"/>
       <c r="H309" s="14"/>
     </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A310" s="16"/>
       <c r="B310" s="15"/>
       <c r="C310" s="15"/>
@@ -6298,7 +6438,7 @@
       <c r="G310" s="56"/>
       <c r="H310" s="14"/>
     </row>
-    <row r="311" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A311" s="16"/>
       <c r="B311" s="15"/>
       <c r="C311" s="15"/>
@@ -6306,7 +6446,7 @@
       <c r="G311" s="56"/>
       <c r="H311" s="14"/>
     </row>
-    <row r="312" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A312" s="16"/>
       <c r="B312" s="15"/>
       <c r="C312" s="15"/>
@@ -6314,7 +6454,7 @@
       <c r="G312" s="56"/>
       <c r="H312" s="14"/>
     </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A313" s="38"/>
       <c r="B313" s="15"/>
       <c r="C313" s="15"/>
@@ -6322,7 +6462,7 @@
       <c r="G313" s="56"/>
       <c r="H313" s="14"/>
     </row>
-    <row r="314" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A314" s="50"/>
       <c r="B314" s="15"/>
       <c r="C314" s="15"/>
@@ -6330,7 +6470,7 @@
       <c r="G314" s="56"/>
       <c r="H314" s="14"/>
     </row>
-    <row r="315" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A315" s="16"/>
       <c r="B315" s="15"/>
       <c r="C315" s="15"/>
@@ -6338,7 +6478,7 @@
       <c r="G315" s="56"/>
       <c r="H315" s="14"/>
     </row>
-    <row r="316" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A316" s="16"/>
       <c r="B316" s="15"/>
       <c r="C316" s="15"/>
@@ -6346,7 +6486,7 @@
       <c r="G316" s="56"/>
       <c r="H316" s="14"/>
     </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A317" s="16"/>
       <c r="B317" s="15"/>
       <c r="C317" s="15"/>
@@ -6354,7 +6494,7 @@
       <c r="G317" s="56"/>
       <c r="H317" s="14"/>
     </row>
-    <row r="318" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A318" s="38"/>
       <c r="B318" s="15"/>
       <c r="C318" s="15"/>
@@ -6362,7 +6502,7 @@
       <c r="G318" s="56"/>
       <c r="H318" s="14"/>
     </row>
-    <row r="319" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A319" s="50"/>
       <c r="B319" s="15"/>
       <c r="C319" s="15"/>
@@ -6370,7 +6510,7 @@
       <c r="G319" s="56"/>
       <c r="H319" s="14"/>
     </row>
-    <row r="320" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A320" s="16"/>
       <c r="B320" s="15"/>
       <c r="C320" s="15"/>
@@ -6378,7 +6518,7 @@
       <c r="G320" s="56"/>
       <c r="H320" s="14"/>
     </row>
-    <row r="321" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A321" s="16"/>
       <c r="B321" s="15"/>
       <c r="C321" s="15"/>
@@ -6386,7 +6526,7 @@
       <c r="G321" s="56"/>
       <c r="H321" s="14"/>
     </row>
-    <row r="322" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A322" s="16"/>
       <c r="B322" s="15"/>
       <c r="C322" s="15"/>
@@ -6394,7 +6534,7 @@
       <c r="G322" s="56"/>
       <c r="H322" s="14"/>
     </row>
-    <row r="323" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A323" s="38"/>
       <c r="B323" s="15"/>
       <c r="C323" s="15"/>
@@ -6402,7 +6542,7 @@
       <c r="G323" s="56"/>
       <c r="H323" s="14"/>
     </row>
-    <row r="324" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A324" s="50"/>
       <c r="B324" s="15"/>
       <c r="C324" s="15"/>
@@ -6410,7 +6550,7 @@
       <c r="G324" s="56"/>
       <c r="H324" s="14"/>
     </row>
-    <row r="325" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A325" s="16"/>
       <c r="B325" s="15"/>
       <c r="C325" s="15"/>
@@ -6418,7 +6558,7 @@
       <c r="G325" s="56"/>
       <c r="H325" s="14"/>
     </row>
-    <row r="326" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A326" s="16"/>
       <c r="B326" s="15"/>
       <c r="C326" s="15"/>
@@ -6426,7 +6566,7 @@
       <c r="G326" s="56"/>
       <c r="H326" s="14"/>
     </row>
-    <row r="327" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A327" s="16"/>
       <c r="B327" s="15"/>
       <c r="C327" s="15"/>
@@ -6434,7 +6574,7 @@
       <c r="G327" s="56"/>
       <c r="H327" s="14"/>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A328" s="38"/>
       <c r="B328" s="15"/>
       <c r="C328" s="15"/>
@@ -6442,7 +6582,7 @@
       <c r="G328" s="56"/>
       <c r="H328" s="14"/>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A329" s="50"/>
       <c r="B329" s="15"/>
       <c r="C329" s="15"/>
@@ -6450,7 +6590,7 @@
       <c r="G329" s="56"/>
       <c r="H329" s="14"/>
     </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A330" s="16"/>
       <c r="B330" s="15"/>
       <c r="C330" s="15"/>
@@ -6458,7 +6598,7 @@
       <c r="G330" s="56"/>
       <c r="H330" s="14"/>
     </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A331" s="16"/>
       <c r="B331" s="15"/>
       <c r="C331" s="15"/>
@@ -6466,7 +6606,7 @@
       <c r="G331" s="56"/>
       <c r="H331" s="14"/>
     </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A332" s="16"/>
       <c r="B332" s="15"/>
       <c r="C332" s="15"/>
@@ -6474,7 +6614,7 @@
       <c r="G332" s="56"/>
       <c r="H332" s="14"/>
     </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A333" s="38"/>
       <c r="B333" s="15"/>
       <c r="C333" s="15"/>
@@ -6482,7 +6622,7 @@
       <c r="G333" s="56"/>
       <c r="H333" s="14"/>
     </row>
-    <row r="334" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A334" s="50"/>
       <c r="B334" s="15"/>
       <c r="C334" s="15"/>
@@ -6490,7 +6630,7 @@
       <c r="G334" s="56"/>
       <c r="H334" s="14"/>
     </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A335" s="16"/>
       <c r="B335" s="15"/>
       <c r="C335" s="15"/>
@@ -6498,7 +6638,7 @@
       <c r="G335" s="56"/>
       <c r="H335" s="14"/>
     </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A336" s="16"/>
       <c r="B336" s="15"/>
       <c r="C336" s="15"/>
@@ -6506,7 +6646,7 @@
       <c r="G336" s="56"/>
       <c r="H336" s="14"/>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A337" s="16"/>
       <c r="B337" s="15"/>
       <c r="C337" s="15"/>
@@ -6514,7 +6654,7 @@
       <c r="G337" s="56"/>
       <c r="H337" s="14"/>
     </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A338" s="38"/>
       <c r="B338" s="15"/>
       <c r="C338" s="15"/>
@@ -6522,7 +6662,7 @@
       <c r="G338" s="56"/>
       <c r="H338" s="14"/>
     </row>
-    <row r="339" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A339" s="50"/>
       <c r="B339" s="15"/>
       <c r="C339" s="15"/>
@@ -6530,7 +6670,7 @@
       <c r="G339" s="56"/>
       <c r="H339" s="14"/>
     </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A340" s="16"/>
       <c r="B340" s="15"/>
       <c r="C340" s="15"/>
@@ -6538,7 +6678,7 @@
       <c r="G340" s="56"/>
       <c r="H340" s="14"/>
     </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A341" s="16"/>
       <c r="B341" s="15"/>
       <c r="C341" s="15"/>
@@ -6546,7 +6686,7 @@
       <c r="G341" s="56"/>
       <c r="H341" s="14"/>
     </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A342" s="16"/>
       <c r="B342" s="15"/>
       <c r="C342" s="15"/>
@@ -6554,7 +6694,7 @@
       <c r="G342" s="56"/>
       <c r="H342" s="14"/>
     </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A343" s="38"/>
       <c r="B343" s="15"/>
       <c r="C343" s="15"/>
@@ -6562,7 +6702,7 @@
       <c r="G343" s="56"/>
       <c r="H343" s="14"/>
     </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A344" s="50"/>
       <c r="B344" s="15"/>
       <c r="C344" s="15"/>
@@ -6570,7 +6710,7 @@
       <c r="G344" s="56"/>
       <c r="H344" s="14"/>
     </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A345" s="16"/>
       <c r="B345" s="15"/>
       <c r="C345" s="15"/>
@@ -6578,7 +6718,7 @@
       <c r="G345" s="56"/>
       <c r="H345" s="14"/>
     </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A346" s="16"/>
       <c r="B346" s="15"/>
       <c r="C346" s="15"/>
@@ -6592,20 +6732,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6616,7 +6756,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -6627,7 +6767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Se añaden parametros nuevos al excel y las funcionalidades para extraerlos
</commit_message>
<xml_diff>
--- a/data/data_electrico_var_3turnos_chuqui_seasons/elmo_data.xlsx
+++ b/data/data_electrico_var_3turnos_chuqui_seasons/elmo_data.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\ELMO-UG-Paper\data\data_electrico_var_3turnos_chuqui_seasons\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB038231-4D14-4B80-9124-8223664FC97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F5B241-6EE7-46D6-B3F2-6DFF9ADCA2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
     <sheet name="LHD" sheetId="2" r:id="rId2"/>
     <sheet name="stations" sheetId="5" r:id="rId3"/>
-    <sheet name="extraction_nodes" sheetId="3" r:id="rId4"/>
-    <sheet name="discharge_nodes" sheetId="4" r:id="rId5"/>
+    <sheet name="chargers" sheetId="6" r:id="rId4"/>
+    <sheet name="extraction_nodes" sheetId="3" r:id="rId5"/>
+    <sheet name="discharge_nodes" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="132">
   <si>
     <t>id</t>
   </si>
@@ -412,6 +413,27 @@
   </si>
   <si>
     <t>station_3</t>
+  </si>
+  <si>
+    <t>charger_model</t>
+  </si>
+  <si>
+    <t>charger_cost</t>
+  </si>
+  <si>
+    <t>charger_power</t>
+  </si>
+  <si>
+    <t>num_connectors</t>
+  </si>
+  <si>
+    <t>Sandvik</t>
+  </si>
+  <si>
+    <t>p_max_dist</t>
+  </si>
+  <si>
+    <t>p_peak_dist</t>
   </si>
 </sst>
 </file>
@@ -2812,6 +2834,90 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0351544-AA63-4F3E-855C-5CF465DCF681}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3">
+        <v>47304</v>
+      </c>
+      <c r="D3">
+        <v>353</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>2100</v>
+      </c>
+      <c r="G3">
+        <v>1500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6732,7 +6838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>

</xml_diff>